<commit_message>
campo origem planilha v2 pudim
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/dados_teste/DADOS_V2_PUDIM.xlsx
+++ b/V. 2 (Pudim)/dados_teste/DADOS_V2_PUDIM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Documents\dev\Finscore\FinScore\V. 2 (Pudim)\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188BB1E4-9F45-4FC0-8888-0BBFE4DE6C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61F23B0-BB91-476C-B7D6-9D132B9212A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="95">
   <si>
     <t>ano</t>
   </si>
@@ -132,9 +132,6 @@
   </si>
   <si>
     <t>r_Despesa_Juros</t>
-  </si>
-  <si>
-    <t>r_Depreciacao_Amortizacao_Exaustão</t>
   </si>
   <si>
     <t>r_EBIT</t>
@@ -275,9 +272,6 @@
     <t>Nome da Conta em Demonstrações Contábeis</t>
   </si>
   <si>
-    <t>Nomes mais comuns nas Demonstrações Contábeis</t>
-  </si>
-  <si>
     <t>Ano, Exercício, Exercício Social, Período, Período de Referência, Data-Base, Encerramento do Exercício</t>
   </si>
   <si>
@@ -384,6 +378,35 @@
   </si>
   <si>
     <t>Caixa e Equivalentes</t>
+  </si>
+  <si>
+    <t>r_Depreciacao_Amortizacao_Exaustao</t>
+  </si>
+  <si>
+    <t>Aquisições de Ativo Imobilizado, Aquisição de Imobilizado, Adições ao Imobilizado, Compras de Imobilizado, Aquisições de Ativo Intangível, Aquisição de Intangível, Adições ao Intangível, Aquisições de Imobilizado e Intangível, Investimentos em Imobilizado e Intangível, Pagamentos pela Aquisição de Imobilizado e Intangível, Gastos de Capital, Dispêndios de Capital, CAPEX</t>
+  </si>
+  <si>
+    <t>Origem</t>
+  </si>
+  <si>
+    <t>Balanço Patrimonial (BP)</t>
+  </si>
+  <si>
+    <t>Notas Explicativas</t>
+  </si>
+  <si>
+    <t>Demonstração do Resultado do Exercício (DRE)</t>
+  </si>
+  <si>
+    <t>Demonstração de Fluxo de Caixa (DFC)
+Notas Explicativas</t>
+  </si>
+  <si>
+    <t>Demonstração do Resultado do Exercício (DRE)
+Notas Explicativas</t>
+  </si>
+  <si>
+    <t>Demonstração de Fluxo de Caixa (DFC)</t>
   </si>
 </sst>
 </file>
@@ -970,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C1" s="25" t="s">
         <v>7</v>
@@ -1009,10 +1032,10 @@
         <v>13</v>
       </c>
       <c r="O1" s="27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P1" s="28" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="Q1" s="28" t="s">
         <v>14</v>
@@ -1021,10 +1044,10 @@
         <v>6</v>
       </c>
       <c r="S1" s="29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T1" s="29" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="U1" s="23"/>
       <c r="V1" s="23"/>
@@ -1063,7 +1086,7 @@
     </row>
     <row r="3" spans="1:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="31"/>
@@ -28020,446 +28043,510 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD9C50DC-59BA-46D6-8542-7646E880A7E2}">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53.44140625" style="7" customWidth="1"/>
     <col min="2" max="2" width="40.6640625" style="6" customWidth="1"/>
     <col min="3" max="3" width="88.6640625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="40.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="62.21875" style="6" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="7"/>
+    <col min="4" max="4" width="36.88671875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="40.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="62.21875" style="6" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>21</v>
+      <c r="C1" s="16" t="s">
+        <v>18</v>
       </c>
-      <c r="C1" s="16" t="s">
-        <v>19</v>
+      <c r="D1" s="16" t="s">
+        <v>88</v>
       </c>
-      <c r="D1" s="15" t="s">
-        <v>61</v>
+      <c r="E1" s="15" t="s">
+        <v>60</v>
       </c>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="D2" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D3" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="7"/>
-    </row>
-    <row r="3" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="E3" s="7"/>
-    </row>
-    <row r="4" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>26</v>
+      <c r="D4" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D4" s="12" t="s">
-        <v>64</v>
+      <c r="E4" s="12" t="s">
+        <v>63</v>
       </c>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>28</v>
+      <c r="D5" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>65</v>
+      <c r="E5" s="12" t="s">
+        <v>64</v>
       </c>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>30</v>
+      <c r="D6" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>66</v>
+      <c r="E6" s="12" t="s">
+        <v>65</v>
       </c>
-      <c r="E6" s="7"/>
-    </row>
-    <row r="7" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>32</v>
+      <c r="D7" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D7" s="12" t="s">
-        <v>67</v>
+      <c r="E7" s="12" t="s">
+        <v>66</v>
       </c>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>34</v>
+      <c r="D8" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D8" s="12" t="s">
-        <v>68</v>
+      <c r="E8" s="12" t="s">
+        <v>67</v>
       </c>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>36</v>
+      <c r="D9" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D9" s="12" t="s">
-        <v>69</v>
+      <c r="E9" s="12" t="s">
+        <v>68</v>
       </c>
-      <c r="E9" s="7"/>
-    </row>
-    <row r="10" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>38</v>
+      <c r="D10" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D10" s="12" t="s">
-        <v>70</v>
+      <c r="E10" s="12" t="s">
+        <v>69</v>
       </c>
-      <c r="E10" s="7"/>
-    </row>
-    <row r="11" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>40</v>
+      <c r="D11" s="12" t="s">
+        <v>89</v>
       </c>
-      <c r="D11" s="12" t="s">
-        <v>71</v>
+      <c r="E11" s="12" t="s">
+        <v>70</v>
       </c>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="12" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:6" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>42</v>
+      <c r="D12" s="12" t="s">
+        <v>90</v>
       </c>
-      <c r="D12" s="12" t="s">
-        <v>72</v>
+      <c r="E12" s="12" t="s">
+        <v>71</v>
       </c>
-      <c r="E12" s="7"/>
-    </row>
-    <row r="13" spans="1:5" ht="96.6" x14ac:dyDescent="0.3">
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:6" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>44</v>
+      <c r="D13" s="12" t="s">
+        <v>90</v>
       </c>
-      <c r="D13" s="12" t="s">
-        <v>73</v>
+      <c r="E13" s="13" t="s">
+        <v>72</v>
       </c>
-      <c r="E13" s="7"/>
-    </row>
-    <row r="14" spans="1:5" ht="96.6" x14ac:dyDescent="0.3">
+      <c r="F13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="13" t="s">
-        <v>46</v>
+      <c r="D14" s="13" t="s">
+        <v>91</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>74</v>
+      <c r="E14" s="13" t="s">
+        <v>73</v>
       </c>
-      <c r="E14" s="7"/>
-    </row>
-    <row r="15" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:6" ht="69" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="D15" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" ht="69" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="C16" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:5" ht="69" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>16</v>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>86</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="13" t="s">
+      <c r="B17" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="C17" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" spans="1:5" ht="69" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="E17" s="7"/>
-    </row>
-    <row r="18" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" ht="69" x14ac:dyDescent="0.3">
       <c r="A18" s="21" t="s">
         <v>14</v>
       </c>
       <c r="B18" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="13" t="s">
-        <v>54</v>
+      <c r="D18" s="13" t="s">
+        <v>93</v>
       </c>
-      <c r="D18" s="13" t="s">
-        <v>78</v>
+      <c r="E18" s="13" t="s">
+        <v>77</v>
       </c>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" ht="69" x14ac:dyDescent="0.3">
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B19" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="D19" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="C20" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="E20" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="1:5" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C20" s="13" t="s">
+      <c r="B21" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="C21" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" s="7"/>
+    </row>
+    <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="7"/>
-    </row>
-    <row r="21" spans="1:5" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="13" t="s">
+    </row>
+    <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="18"/>
+    </row>
+    <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="23" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="17" t="s">
+    </row>
+    <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="19" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="18"/>
-    </row>
-    <row r="25" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="19" t="s">
+      <c r="B26" s="7"/>
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="19" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="B26" s="7"/>
-      <c r="E26" s="7"/>
-    </row>
-    <row r="27" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="19" t="s">
-        <v>85</v>
-      </c>
       <c r="B27" s="7"/>
-      <c r="E27" s="7"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B28" s="7"/>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B29" s="7"/>
-      <c r="E29" s="7"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" s="7"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B30" s="7"/>
-      <c r="E30" s="7"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="7"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B31" s="7"/>
-      <c r="E31" s="7"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B32" s="7"/>
-      <c r="E32" s="7"/>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="7"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7"/>
-      <c r="E33" s="7"/>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F33" s="7"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="7"/>
-      <c r="E34" s="7"/>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F34" s="7"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" s="7"/>
-      <c r="E35" s="7"/>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F35" s="7"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" s="7"/>
-      <c r="E36" s="7"/>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F36" s="7"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" s="7"/>
-      <c r="E37" s="7"/>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F37" s="7"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="7"/>
-      <c r="E38" s="7"/>
-    </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F38" s="7"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B39" s="7"/>
-      <c r="E39" s="7"/>
-    </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B40" s="7"/>
-      <c r="E40" s="7"/>
-    </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F40" s="7"/>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B41" s="7"/>
-      <c r="E41" s="7"/>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F41" s="7"/>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B42" s="7"/>
-      <c r="E42" s="7"/>
-    </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F42" s="7"/>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="7"/>
-      <c r="E43" s="7"/>
-    </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F43" s="7"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B44" s="7"/>
-      <c r="E44" s="7"/>
-    </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F44" s="7"/>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B45" s="7"/>
-      <c r="E45" s="7"/>
-    </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F45" s="7"/>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B46" s="7"/>
-      <c r="E46" s="7"/>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F46" s="7"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B47" s="7"/>
-      <c r="E47" s="7"/>
-    </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F47" s="7"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B48" s="7"/>
-      <c r="E48" s="7"/>
-    </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F48" s="7"/>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B49" s="7"/>
-      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
análise crítica das contas da planilha das contas
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/dados_teste/DADOS_V2_PUDIM.xlsx
+++ b/V. 2 (Pudim)/dados_teste/DADOS_V2_PUDIM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Documents\dev\Finscore\FinScore\V. 2 (Pudim)\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61F23B0-BB91-476C-B7D6-9D132B9212A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{949381DB-D16A-4D44-BA90-C34864139042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -413,7 +413,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -518,6 +518,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -602,7 +608,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -700,6 +706,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -28253,41 +28268,39 @@
       </c>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" ht="96.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:6" s="35" customFormat="1" ht="96.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="F12" s="7"/>
-    </row>
-    <row r="13" spans="1:6" ht="96.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:6" s="35" customFormat="1" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="7"/>
     </row>
     <row r="14" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
@@ -28343,41 +28356,39 @@
       </c>
       <c r="F16" s="7"/>
     </row>
-    <row r="17" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" s="35" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="7"/>
-    </row>
-    <row r="18" spans="1:6" ht="69" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:6" s="35" customFormat="1" ht="69" x14ac:dyDescent="0.3">
       <c r="A18" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
@@ -28415,23 +28426,22 @@
       </c>
       <c r="F20" s="7"/>
     </row>
-    <row r="21" spans="1:6" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" s="35" customFormat="1" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="7"/>
     </row>
     <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">

</xml_diff>